<commit_message>
fullgame/FG-M0: FG0-ARCH-01 整个世界同时运行与统一时钟底座 Completed
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/fg/#HomeTuning-家园与格网调参.xlsx
+++ b/Configs/GameConfig/Datas/fg/#HomeTuning-家园与格网调参.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1058,6 +1058,246 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>clock.sim_step_hz</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>60</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>世界模拟固定步长频率(次/游戏秒);与渲染帧率无关,倍速只改变每帧跑几步,结果与1x一致</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>clock.max_steps_per_frame</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>12</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>单帧最多补跑的模拟步数(防卡顿雪崩);超出部分丢弃=世界短暂变慢,不跳步</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>clock.max_frame_seconds</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>单帧计入的真实时间上限(秒);断点/加载后的超长帧不会一次补跑几十秒</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>clock.day_seconds</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1个游戏日在1x下的真实秒数(FGR-ENV-001:20分钟;1游戏小时=50秒)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>clock.start_hour</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>6</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>新战役开始时是当天几点(0~23),第1日从这个时刻起算</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>clock.objective_recompute_seconds</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>目标兜底重算间隔(游戏秒,跟随世界模拟步进,观察与否一致)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>sim.activity_refresh_seconds</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>活跃区块集合(己方实体/行进中的队伍/被观察)重算间隔(游戏秒)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>camera.fly_seconds</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>镜头飞跃过渡时长(真实秒),FG17 初值 0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>camera.explored_margin_cells</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>24</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>星球镜头可平移范围=已探索区域外再放宽多少格</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>camera.precision_safe_cells</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>16384</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>不启用浮动原点时镜头可达范围上限(格);超出前必须接浮动原点(DEBT-FG0ARCH01-02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>camera.zoom_min_ortho</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>8</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>战略视角最近缩放(正交半高,格);Demo 初值 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>camera.zoom_max_ortho</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>46</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>战略视角最远缩放(正交半高,格);整个已探索世界的战略地图缩放由 FG17 FGR-GEN-080 承接卡放宽(DEBT-FG0ARCH01-08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>camera.zoom_step</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>鼠标滚轮每格的缩放量(正交半高,格)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>transit.raid_speed_cells_per_second</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>突袭队伍在星球上的行进速度(格/游戏秒);FG6-DEF-04 起按编成里最慢的单位取</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>transit.arrival_radius_cells</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>12</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>队伍离目标多少格以内算到达</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fullgame/FG-M0: FG0-ARCH-02 传送带内核原型 Completed
Main/Sim/Logistics 传送带内核（BeltKernel/BeltJobs/BeltRenderer/BeltTypes）+ 热更侧
BeltNetworkService 接入；修复轮解决环上侧向汇入卡死、车道跨格间距、格式版本通知、
远景重填、端口名读档丢失等问题；新增自检 FgBeltKernelSelfCheck 与渲染探针
FgBeltRenderProbe；GameRes 指针随导表数据更新。

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/fg/#HomeTuning-家园与格网调参.xlsx
+++ b/Configs/GameConfig/Datas/fg/#HomeTuning-家园与格网调参.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1298,6 +1298,166 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>logistics.step_hz</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>20</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>传送带内核固定步长频率(次/游戏秒),FGR-ARC-004 初值 20;在 60Hz 世界步里按游戏时间累计推进</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>logistics.slots_per_cell</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>4</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>每格传送带最多几个物品(1~4),FG03 第10章初值 4;物品最小间距=1/该值 格</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>logistics.items_per_minute_t1</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>60</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>T1 传送带满载吞吐(件/分钟),FG03 第10章初值</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>logistics.items_per_minute_t2</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>120</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>T2 传送带满载吞吐(件/分钟)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>logistics.items_per_minute_t3</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>240</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>T3 传送带满载吞吐(件/分钟)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>logistics.stats_bucket_steps</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>300</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>吞吐统计快照间隔(内核步);窗口=4个快照(20Hz 下 60 游戏秒)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>logistics.render.flow_ortho_enter</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>38</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>镜头正交半高 &gt;= 此值切到远景流动贴图(不再逐物品绘制);须大于家园默认缩放 30、小于最远 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>logistics.render.flow_ortho_exit</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>34</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>远景下正交半高 &lt;= 此值切回近景(回差,避免在阈值附近来回闪)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>logistics.render.item_size</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>带上物品的边长(格)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>logistics.render.height</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>传送带面的高度(世界单位,在地貌之上、建筑之下)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fullgame/FG-M0: FG0-ARCH-03 战斗内核接入 Completed
新增 Main/Sim/Combat 战斗内核（单线程 Burst，确定性）与热更侧 Campaign/Combat 桥接层（20 个门面方法）；
删除 Demo 的 CannonCombat/FracturedCityEnemyAi/FoundryOutpostEnemyAi；机器表现改逻辑句柄 + ViewMaterials 材质共享。
修复审查 3 条 P1：存档写回前排空积压阵亡事件、切换观察泄漏材质、9 个热更文件绕过桥接层直调内核。

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/fg/#HomeTuning-家园与格网调参.xlsx
+++ b/Configs/GameConfig/Datas/fg/#HomeTuning-家园与格网调参.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1458,6 +1458,518 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>combat.grid_cell_m</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>8</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>战斗内核空间网格格边长(米);目标选择与弹体碰撞按格查询,结果只由比较规则决定(确定性)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>combat.events.gameplay_per_step</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>64</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>每个地点每步最多交给热更层处理的玩法事件数(阵亡/伤害请求/命令结束等);超出的留到下一步,永不丢弃,进存档</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>combat.events.cues_per_step</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>24</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>每个地点每步最多保留的提示事件数(开火音/护甲命中等);超出的丢弃并计数(B17 同类音效有数量上限)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>combat.projectile_capacity</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>4096</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>每个地点同时存在的弹体上限;超出的开火不生成弹体并计数(FGR-SYS-041 目标 1500)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>combat.compact_ratio</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>阵亡即移除的单位占槽位比例超过此值时在步首压实(保持相对顺序)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>combat.render.unit_height</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>实例化单位(突袭者/炮塔原型)圆片的画面高度(世界单位)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>combat.bench.raider_hp</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>120</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>突袭者原型耐久</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>combat.bench.raider_speed</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>突袭者原型移动速度(米/游戏秒)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>combat.bench.raider_radius</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>突袭者原型半径(米)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>combat.bench.raider_sense</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>60</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>突袭者原型感知距离(米):范围内有己方目标就扑过去,否则朝目标点前进</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>combat.bench.raider_range</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>16</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>突袭者原型射程(米)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>combat.bench.raider_damage</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>6</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>突袭者原型每发伤害</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>combat.bench.raider_cooldown</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>突袭者原型开火间隔(游戏秒)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>combat.bench.raider_projectile_speed</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>18</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>突袭者原型弹速(米/游戏秒)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>combat.bench.raider_projectile_radius</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>突袭者原型弹体半径(米)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr"/>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>combat.bench.turret_hp</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>400</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>炮塔原型耐久</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr"/>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>combat.bench.turret_radius</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>炮塔原型半径(米,轻型 2x2 占地的内切圆)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>combat.bench.turret_range</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>26</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>炮塔原型射程(米)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr"/>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>combat.bench.turret_damage</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>14</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>炮塔原型每发伤害</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr"/>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>combat.bench.turret_cooldown</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>炮塔原型开火间隔(游戏秒)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr"/>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>combat.bench.turret_projectile_speed</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>24</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>炮塔原型弹速(米/游戏秒)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr"/>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>combat.bench.turret_projectile_radius</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>炮塔原型弹体半径(米)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr"/>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>combat.perf.enemies</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>200</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>性能场景:同时存在的敌人数</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr"/>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>combat.perf.turrets</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>80</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>性能场景:炮塔数</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr"/>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>combat.perf.min_projectiles</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>性能场景:测量窗口内同时存在的弹体数下限</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr"/>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>combat.perf.step_budget_ms</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>6</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>战斗内核单步预算(毫秒,推荐配置;FGR-SYS-042 内核(物流+战斗)&lt;=6ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr"/>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>combat.perf.hp_scale</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>25</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>性能场景:突袭者与炮塔耐久倍率(让测量窗口内双方数量保持在规模目标附近)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr"/>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>combat.perf.turret_cooldown</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>性能场景:炮塔开火间隔(游戏秒)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr"/>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>combat.perf.raider_cooldown</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>性能场景:突袭者开火间隔(游戏秒)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr"/>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>combat.perf.projectile_speed</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>8</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>性能场景:弹速(米/游戏秒;较慢,让弹体在空中停留更久,达到同时存在的弹体数目标)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr"/>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>combat.perf.turret_range</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>30</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>性能场景:炮塔射程(米)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr"/>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>combat.perf.raider_range</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>20</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>性能场景:突袭者射程(米)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fullgame/FG-M1: FG1-HUD-01 接入 HUD、机器经历与引导钩子
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/fg/#HomeTuning-家园与格网调参.xlsx
+++ b/Configs/GameConfig/Datas/fg/#HomeTuning-家园与格网调参.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D157"/>
+  <dimension ref="A1:D160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2742,15 +2742,15 @@
       <c r="A145" t="inlineStr"/>
       <c r="B145" t="inlineStr">
         <is>
-          <t>signal.raw.charge_interval_seconds</t>
+          <t>signal.link.strength_full_cells</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>常规裸跑固件的“发动”计次间隔(游戏秒):武器开火即发动一次并计暴露,之后这么久内的开火不再计(与核心固件冷却同初值;记在信号上,换机器不重置,进存档)</t>
+          <t>接入 HUD 链路强度满格所需的离覆盖边缘格数(补全项:FG01 只写“越近越弱”;60 = 预警距离 15 的 4 倍)</t>
         </is>
       </c>
     </row>
@@ -2758,15 +2758,15 @@
       <c r="A146" t="inlineStr"/>
       <c r="B146" t="inlineStr">
         <is>
-          <t>exposure.max</t>
+          <t>signal.link.strength_strong_percent</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>信号暴露上限(沿用 Demo 0～100)</t>
+          <t>链路强度不低于这个百分比显示“强”</t>
         </is>
       </c>
     </row>
@@ -2774,15 +2774,15 @@
       <c r="A147" t="inlineStr"/>
       <c r="B147" t="inlineStr">
         <is>
-          <t>exposure.core_fire</t>
+          <t>signal.link.strength_medium_percent</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>0.5</v>
+        <v>34</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>核心固件每次发动增加的暴露(FG16 初值 +0.5;“发动”= 具名反应真正打出的那一发,FG1-SIG-03)</t>
+          <t>链路强度不低于这个百分比显示“中”,再低显示“弱”;进入边缘预警时显示“边缘”</t>
         </is>
       </c>
     </row>
@@ -2790,15 +2790,15 @@
       <c r="A148" t="inlineStr"/>
       <c r="B148" t="inlineStr">
         <is>
-          <t>exposure.high_power.threshold</t>
+          <t>signal.raw.charge_interval_seconds</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>高功率生产:家园总用电需求超过这个值的部分才计暴露(补全项:FG16 只写“按总功率换算”,阈值 = Demo 开局满配供电 20+80)</t>
+          <t>常规裸跑固件的“发动”计次间隔(游戏秒):武器开火即发动一次并计暴露,之后这么久内的开火不再计(与核心固件冷却同初值;记在信号上,换机器不重置,进存档)</t>
         </is>
       </c>
     </row>
@@ -2806,15 +2806,15 @@
       <c r="A149" t="inlineStr"/>
       <c r="B149" t="inlineStr">
         <is>
-          <t>exposure.high_power.full_at</t>
+          <t>exposure.max</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>高功率生产:总用电需求达到这个值时按每游戏小时上限计;阈值到这里之间线性</t>
+          <t>信号暴露上限(沿用 Demo 0～100)</t>
         </is>
       </c>
     </row>
@@ -2822,15 +2822,15 @@
       <c r="A150" t="inlineStr"/>
       <c r="B150" t="inlineStr">
         <is>
-          <t>exposure.high_power.cap_per_hour</t>
+          <t>exposure.core_fire</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>高功率生产每游戏小时最多增加的暴露(FG16 初值 +3;按游戏时间累计,家园不被观察时照常)</t>
+          <t>核心固件每次发动增加的暴露(FG16 初值 +0.5;“发动”= 具名反应真正打出的那一发,FG1-SIG-03)</t>
         </is>
       </c>
     </row>
@@ -2838,15 +2838,15 @@
       <c r="A151" t="inlineStr"/>
       <c r="B151" t="inlineStr">
         <is>
-          <t>exposure.high_power.settle_seconds</t>
+          <t>exposure.high_power.threshold</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>高功率生产的结算间隔(游戏秒;50 = 1 游戏小时,每小时记一笔来源,不逐帧刷明细)</t>
+          <t>高功率生产:家园总用电需求超过这个值的部分才计暴露(补全项:FG16 只写“按总功率换算”,阈值 = Demo 开局满配供电 20+80)</t>
         </is>
       </c>
     </row>
@@ -2854,15 +2854,15 @@
       <c r="A152" t="inlineStr"/>
       <c r="B152" t="inlineStr">
         <is>
-          <t>exposure.alien_tech_per_expedition</t>
+          <t>exposure.high_power.full_at</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>使用异派技术:出发的远征队里有机器装着跨阵营蓝图时,每次远征 +2(FG16 初值;取代 Demo“首次使用异派固件 +10”)</t>
+          <t>高功率生产:总用电需求达到这个值时按每游戏小时上限计;阈值到这里之间线性</t>
         </is>
       </c>
     </row>
@@ -2870,7 +2870,7 @@
       <c r="A153" t="inlineStr"/>
       <c r="B153" t="inlineStr">
         <is>
-          <t>exposure.node_destroyed</t>
+          <t>exposure.high_power.cap_per_hour</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -2878,7 +2878,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>摧毁敌方节点每个 +3(FG16 初值;取代 Demo 战斗 +8)</t>
+          <t>高功率生产每游戏小时最多增加的暴露(FG16 初值 +3;按游戏时间累计,家园不被观察时照常)</t>
         </is>
       </c>
     </row>
@@ -2886,15 +2886,15 @@
       <c r="A154" t="inlineStr"/>
       <c r="B154" t="inlineStr">
         <is>
-          <t>exposure.node_link_cut_drop</t>
+          <t>exposure.high_power.settle_seconds</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>摧毁监听节点切断监听链,暴露降低这么多(沿用 Demo 的降暴露手段 -15;调参表只收正数,代码里取负)</t>
+          <t>高功率生产的结算间隔(游戏秒;50 = 1 游戏小时,每小时记一笔来源,不逐帧刷明细)</t>
         </is>
       </c>
     </row>
@@ -2902,7 +2902,7 @@
       <c r="A155" t="inlineStr"/>
       <c r="B155" t="inlineStr">
         <is>
-          <t>exposure.tower_off_drop_per_10s</t>
+          <t>exposure.alien_tech_per_expedition</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>关闭信号塔主动广播,每 10 游戏秒暴露降低这么多(沿用 Demo 的降暴露手段 -2;代码里取负)</t>
+          <t>使用异派技术:出发的远征队里有机器装着跨阵营蓝图时,每次远征 +2(FG16 初值;取代 Demo“首次使用异派固件 +10”)</t>
         </is>
       </c>
     </row>
@@ -2918,15 +2918,15 @@
       <c r="A156" t="inlineStr"/>
       <c r="B156" t="inlineStr">
         <is>
-          <t>exposure.history_max</t>
+          <t>exposure.node_destroyed</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>64</v>
+        <v>3</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>暴露来源明细最多保留几条(最近的;各来源与各阵营的累计另有汇总,不随明细截断丢失)</t>
+          <t>摧毁敌方节点每个 +3(FG16 初值;取代 Demo 战斗 +8)</t>
         </is>
       </c>
     </row>
@@ -2934,13 +2934,61 @@
       <c r="A157" t="inlineStr"/>
       <c r="B157" t="inlineStr">
         <is>
+          <t>exposure.node_link_cut_drop</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>15</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>摧毁监听节点切断监听链,暴露降低这么多(沿用 Demo 的降暴露手段 -15;调参表只收正数,代码里取负)</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr"/>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>exposure.tower_off_drop_per_10s</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>2</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>关闭信号塔主动广播,每 10 游戏秒暴露降低这么多(沿用 Demo 的降暴露手段 -2;代码里取负)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr"/>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>exposure.history_max</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>64</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>暴露来源明细最多保留几条(最近的;各来源与各阵营的累计另有汇总,不随明细截断丢失)</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr"/>
+      <c r="B160" t="inlineStr">
+        <is>
           <t>morph.transition_seconds</t>
         </is>
       </c>
-      <c r="C157" t="n">
+      <c r="C160" t="n">
         <v>0.3</v>
       </c>
-      <c r="D157" t="inlineStr">
+      <c r="D160" t="inlineStr">
         <is>
           <t>机身形变过渡秒数(FGR-FW-021 初值 0.3;接入与离开都播放、完全可逆;按真实时间计,不随倍速,战略暂停中不走,与接入过渡同一口径)</t>
         </is>

</xml_diff>